<commit_message>
Price List Generator Change
</commit_message>
<xml_diff>
--- a/PythonProjects/marania_invoice_venv/MaraniaOfficeAutomation_Backlog.xlsx
+++ b/PythonProjects/marania_invoice_venv/MaraniaOfficeAutomation_Backlog.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\GitHub\PythonProjects\marania_invoice_venv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF26D2D3-1C67-43FF-8F58-87D1B5FC0FDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D5A9A9B-EAE7-419F-B820-9E09FAEAB530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{CB46D3C7-3BD4-4495-A761-25302D270CAE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="1" xr2:uid="{CB46D3C7-3BD4-4495-A761-25302D270CAE}"/>
   </bookViews>
   <sheets>
     <sheet name="MaraniaOfficeAutoation-Backlog" sheetId="1" r:id="rId1"/>
+    <sheet name="Modulewise_Backlo" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="78">
   <si>
     <t>#</t>
   </si>
@@ -159,13 +160,127 @@
   </si>
   <si>
     <t>P&amp;L  -in house material value is wrong fix needed</t>
+  </si>
+  <si>
+    <t>Backup</t>
+  </si>
+  <si>
+    <t>All Module Import &amp; Export</t>
+  </si>
+  <si>
+    <t>CRITICAL</t>
+  </si>
+  <si>
+    <t>Login</t>
+  </si>
+  <si>
+    <t>User Management</t>
+  </si>
+  <si>
+    <t>PartyRole</t>
+  </si>
+  <si>
+    <t>Parties</t>
+  </si>
+  <si>
+    <t>Transportation</t>
+  </si>
+  <si>
+    <t>Materials</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>PriceCatalog</t>
+  </si>
+  <si>
+    <t>CustomerPriceCatalog</t>
+  </si>
+  <si>
+    <t>CompanySettings</t>
+  </si>
+  <si>
+    <t>Configuration</t>
+  </si>
+  <si>
+    <t>Invoice</t>
+  </si>
+  <si>
+    <t>InvoiceItem</t>
+  </si>
+  <si>
+    <t>Order</t>
+  </si>
+  <si>
+    <t>OrderSpecification</t>
+  </si>
+  <si>
+    <t>ProfitLoss</t>
+  </si>
+  <si>
+    <t>TwineInventory</t>
+  </si>
+  <si>
+    <t>ExcelSheet</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>PaymentReceipt</t>
+  </si>
+  <si>
+    <t>PaymentAllocation</t>
+  </si>
+  <si>
+    <t>OpeningBalance</t>
+  </si>
+  <si>
+    <t>MaterialConversionRatio</t>
+  </si>
+  <si>
+    <t>ProcessingCost</t>
+  </si>
+  <si>
+    <t>MachineOperationalCost</t>
+  </si>
+  <si>
+    <t>AdditionalCost</t>
+  </si>
+  <si>
+    <t>Production</t>
+  </si>
+  <si>
+    <t>ProfitAnalytics</t>
+  </si>
+  <si>
+    <t>PieceWeightAnalyser</t>
+  </si>
+  <si>
+    <t>SettlementInvoice</t>
+  </si>
+  <si>
+    <t>Open Issue Exist?</t>
+  </si>
+  <si>
+    <t>Issue List:</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>NO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -173,8 +288,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -193,8 +315,13 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -251,11 +378,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -275,8 +429,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Bad" xfId="1" builtinId="27"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -862,42 +1023,96 @@
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C15" s="11">
+        <v>10</v>
+      </c>
+      <c r="D15" t="s">
+        <v>40</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15" t="s">
+        <v>41</v>
+      </c>
+      <c r="H15" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="I15" s="12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C16" s="11">
+        <v>11</v>
+      </c>
+      <c r="D16" t="s">
+        <v>43</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C17" s="11">
+        <v>12</v>
+      </c>
+      <c r="D17" t="s">
+        <v>44</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25" spans="3:9" x14ac:dyDescent="0.25">
       <c r="D25" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="3:9" x14ac:dyDescent="0.25">
       <c r="D26" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:9" x14ac:dyDescent="0.25">
       <c r="D27" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="28" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:9" x14ac:dyDescent="0.25">
       <c r="D28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="3:9" x14ac:dyDescent="0.25">
       <c r="D29" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="30" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="3:9" x14ac:dyDescent="0.25">
       <c r="D30" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="31" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="3:9" x14ac:dyDescent="0.25">
       <c r="D31" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="32" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="3:9" x14ac:dyDescent="0.25">
       <c r="D32" t="s">
         <v>39</v>
       </c>
@@ -909,4 +1124,383 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2176B721-3936-4756-811F-AA5B6DEF1B5A}">
+  <dimension ref="B2:F33"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B2" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B3" s="13">
+        <v>1</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B4" s="13">
+        <v>2</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B5" s="13">
+        <v>3</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="13">
+        <v>4</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B7" s="13">
+        <v>5</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B8" s="13">
+        <v>6</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B9" s="13">
+        <v>7</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B10" s="13">
+        <v>8</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B11" s="13">
+        <v>9</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B12" s="13">
+        <v>10</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B13" s="13">
+        <v>11</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B14" s="13">
+        <v>12</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B15" s="13">
+        <v>13</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B16" s="13">
+        <v>14</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B17" s="13">
+        <v>15</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B18" s="13">
+        <v>16</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B19" s="13">
+        <v>17</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B20" s="13">
+        <v>18</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B21" s="13">
+        <v>19</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B22" s="13">
+        <v>20</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B23" s="13">
+        <v>21</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B24" s="13">
+        <v>22</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B25" s="13">
+        <v>23</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="F25" s="13" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B26" s="13">
+        <v>24</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B27" s="13">
+        <v>25</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B28" s="13">
+        <v>26</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="D28" s="13"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="13"/>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B29" s="13">
+        <v>27</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="13"/>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B30" s="13">
+        <v>28</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
+      <c r="F30" s="13"/>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B31" s="13">
+        <v>29</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="13"/>
+    </row>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B32" s="13">
+        <v>30</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="D32" s="13"/>
+      <c r="E32" s="13"/>
+      <c r="F32" s="13"/>
+    </row>
+    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C33" s="14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
login window changes. we may need to comment this if required. CAUTION.
</commit_message>
<xml_diff>
--- a/PythonProjects/marania_invoice_venv/MaraniaOfficeAutomation_Backlog.xlsx
+++ b/PythonProjects/marania_invoice_venv/MaraniaOfficeAutomation_Backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\GitHub\PythonProjects\marania_invoice_venv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D5A9A9B-EAE7-419F-B820-9E09FAEAB530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2774885D-2DFE-4690-9D58-36A35B4D8D14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="1" xr2:uid="{CB46D3C7-3BD4-4495-A761-25302D270CAE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{CB46D3C7-3BD4-4495-A761-25302D270CAE}"/>
   </bookViews>
   <sheets>
     <sheet name="MaraniaOfficeAutoation-Backlog" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="90">
   <si>
     <t>#</t>
   </si>
@@ -274,13 +274,49 @@
   </si>
   <si>
     <t>NO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If possible have a combined price list grouped one </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove unwanted fields like minimum size from admin </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sagar - SI to expense - check </t>
+  </si>
+  <si>
+    <t>Sales - pending delivery date, paid payment date and allocation payment to affect the status</t>
+  </si>
+  <si>
+    <t>1. Twine Inventory - refresh button</t>
+  </si>
+  <si>
+    <t>2. Profit &amp; Loss - refresh button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. how "In-House Material Value (Rs)" value calculated </t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. sales moduel, can we have "S.Edit", ie, selected edit. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. for currency amount, display the comma to easily identify the digit. </t>
+  </si>
+  <si>
+    <t>7. Analytics - group by customers who gave orders monthly wise</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>4. sales module, if invoice number is entered and its in-processing state and delivery date is empty,  fill the values -</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -295,8 +331,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -318,6 +361,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -405,9 +453,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -420,6 +469,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -429,15 +482,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Bad" xfId="1" builtinId="27"/>
+    <cellStyle name="Good" xfId="2" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -770,7 +818,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3105E945-C1D5-4802-BFC4-8648EC86A18C}">
-  <dimension ref="C1:I32"/>
+  <dimension ref="C1:I42"/>
   <sheetFormatPr defaultColWidth="12.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="22.7109375" bestFit="1" customWidth="1"/>
@@ -887,7 +935,7 @@
       <c r="C7" s="3">
         <v>5</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="12" t="s">
         <v>15</v>
       </c>
       <c r="E7" s="4">
@@ -906,7 +954,7 @@
     </row>
     <row r="8" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C8" s="3"/>
-      <c r="D8" s="9"/>
+      <c r="D8" s="13"/>
       <c r="E8">
         <v>2</v>
       </c>
@@ -919,7 +967,7 @@
     </row>
     <row r="9" spans="3:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C9" s="3"/>
-      <c r="D9" s="10"/>
+      <c r="D9" s="14"/>
       <c r="E9" s="5">
         <v>3</v>
       </c>
@@ -1024,7 +1072,7 @@
       </c>
     </row>
     <row r="15" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C15" s="11">
+      <c r="C15" s="3">
         <v>10</v>
       </c>
       <c r="D15" t="s">
@@ -1036,15 +1084,15 @@
       <c r="F15" t="s">
         <v>41</v>
       </c>
-      <c r="H15" s="12" t="s">
+      <c r="H15" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="I15" s="12" t="s">
+      <c r="I15" s="8" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="16" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C16" s="11">
+      <c r="C16" s="3">
         <v>11</v>
       </c>
       <c r="D16" t="s">
@@ -1061,7 +1109,7 @@
       </c>
     </row>
     <row r="17" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C17" s="11">
+      <c r="C17" s="3">
         <v>12</v>
       </c>
       <c r="D17" t="s">
@@ -1077,44 +1125,117 @@
         <v>28</v>
       </c>
     </row>
+    <row r="22" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="D22" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="D23" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="D24" t="s">
+        <v>33</v>
+      </c>
+    </row>
     <row r="25" spans="3:9" x14ac:dyDescent="0.25">
       <c r="D25" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="26" spans="3:9" x14ac:dyDescent="0.25">
       <c r="D26" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="27" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C27" s="11" t="s">
+        <v>88</v>
+      </c>
       <c r="D27" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="28" spans="3:9" x14ac:dyDescent="0.25">
       <c r="D28" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="29" spans="3:9" x14ac:dyDescent="0.25">
       <c r="D29" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="30" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="D30" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="31" spans="3:9" x14ac:dyDescent="0.25">
       <c r="D31" t="s">
-        <v>38</v>
+        <v>78</v>
       </c>
     </row>
     <row r="32" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C32" s="11" t="s">
+        <v>88</v>
+      </c>
       <c r="D32" t="s">
-        <v>39</v>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="33" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C33" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D33" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="34" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C34" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D34" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="36" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C36" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D36" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="37" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D37" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="38" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D38" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="39" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C39" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D39" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="40" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D40" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="41" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D41" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="42" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="D42" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -1137,366 +1258,366 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="9" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="13">
+      <c r="B3" s="9">
         <v>1</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="13">
+      <c r="B4" s="9">
         <v>2</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="13">
+      <c r="B5" s="9">
         <v>3</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="13">
+      <c r="B6" s="9">
         <v>4</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="13">
+      <c r="B7" s="9">
         <v>5</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="13">
+      <c r="B8" s="9">
         <v>6</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="13">
+      <c r="B9" s="9">
         <v>7</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B10" s="13">
+      <c r="B10" s="9">
         <v>8</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B11" s="13">
+      <c r="B11" s="9">
         <v>9</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B12" s="13">
+      <c r="B12" s="9">
         <v>10</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B13" s="13">
+      <c r="B13" s="9">
         <v>11</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="13">
+      <c r="B14" s="9">
         <v>12</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B15" s="13">
+      <c r="B15" s="9">
         <v>13</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B16" s="13">
+      <c r="B16" s="9">
         <v>14</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B17" s="13">
+      <c r="B17" s="9">
         <v>15</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="C17" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B18" s="13">
+      <c r="B18" s="9">
         <v>16</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B19" s="13">
+      <c r="B19" s="9">
         <v>17</v>
       </c>
-      <c r="C19" s="13" t="s">
+      <c r="C19" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="D19" s="13" t="s">
+      <c r="D19" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="E19" s="13" t="s">
+      <c r="E19" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="F19" s="13" t="s">
+      <c r="F19" s="9" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B20" s="13">
+      <c r="B20" s="9">
         <v>18</v>
       </c>
-      <c r="C20" s="13" t="s">
+      <c r="C20" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B21" s="13">
+      <c r="B21" s="9">
         <v>19</v>
       </c>
-      <c r="C21" s="13" t="s">
+      <c r="C21" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B22" s="13">
+      <c r="B22" s="9">
         <v>20</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B23" s="13">
+      <c r="B23" s="9">
         <v>21</v>
       </c>
-      <c r="C23" s="13" t="s">
+      <c r="C23" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B24" s="13">
+      <c r="B24" s="9">
         <v>22</v>
       </c>
-      <c r="C24" s="13" t="s">
+      <c r="C24" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B25" s="13">
+      <c r="B25" s="9">
         <v>23</v>
       </c>
-      <c r="C25" s="13" t="s">
+      <c r="C25" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="D25" s="13" t="s">
+      <c r="D25" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="E25" s="13" t="s">
+      <c r="E25" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="F25" s="13" t="s">
+      <c r="F25" s="9" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B26" s="13">
+      <c r="B26" s="9">
         <v>24</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="C26" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="13"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B27" s="13">
+      <c r="B27" s="9">
         <v>25</v>
       </c>
-      <c r="C27" s="13" t="s">
+      <c r="C27" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B28" s="13">
+      <c r="B28" s="9">
         <v>26</v>
       </c>
-      <c r="C28" s="13" t="s">
+      <c r="C28" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="13"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B29" s="13">
+      <c r="B29" s="9">
         <v>27</v>
       </c>
-      <c r="C29" s="13" t="s">
+      <c r="C29" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="13"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="9"/>
+      <c r="F29" s="9"/>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B30" s="13">
+      <c r="B30" s="9">
         <v>28</v>
       </c>
-      <c r="C30" s="13" t="s">
+      <c r="C30" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="13"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B31" s="13">
+      <c r="B31" s="9">
         <v>29</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="C31" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="13"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="9"/>
+      <c r="F31" s="9"/>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B32" s="13">
+      <c r="B32" s="9">
         <v>30</v>
       </c>
-      <c r="C32" s="13" t="s">
+      <c r="C32" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9"/>
     </row>
     <row r="33" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C33" s="14" t="s">
+      <c r="C33" s="10" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>